<commit_message>
Correct license and map legend
</commit_message>
<xml_diff>
--- a/data/LanguageFamily.xlsx
+++ b/data/LanguageFamily.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/psav050/Documents/GitHub/manyvoices3/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFB03B3-4457-3D46-BDD8-D5997DE4E91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F6D545-9CE5-964B-A66A-915D75F4814F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1360" yWindow="760" windowWidth="28000" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="1280" windowWidth="13220" windowHeight="16460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Many Voices 2 languages" sheetId="7" r:id="rId1"/>
@@ -150,12 +150,6 @@
     <t>English [Gold Coast]</t>
   </si>
   <si>
-    <t>Italian (Rome)</t>
-  </si>
-  <si>
-    <t>Italian (Padua)</t>
-  </si>
-  <si>
     <t>Czech</t>
   </si>
   <si>
@@ -163,6 +157,12 @@
   </si>
   <si>
     <t>Mandarin Chinese [Reading]</t>
+  </si>
+  <si>
+    <t>Italian</t>
+  </si>
+  <si>
+    <t>Spanish</t>
   </si>
 </sst>
 </file>
@@ -371,9 +371,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -393,6 +390,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -677,17 +677,17 @@
     </row>
     <row r="2" spans="1:44" ht="13" x14ac:dyDescent="0.15"/>
     <row r="3" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="G3" s="28" t="s">
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="G3" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
     </row>
     <row r="4" spans="1:44" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
@@ -708,17 +708,17 @@
         <v>21</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I4" s="17"/>
       <c r="J4" s="19"/>
     </row>
     <row r="5" spans="1:44" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
       <c r="D5" s="12">
         <v>11</v>
       </c>
@@ -754,12 +754,12 @@
       <c r="F6" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="28" t="s">
+      <c r="G6" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="28"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="36"/>
     </row>
     <row r="7" spans="1:44" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
@@ -773,41 +773,41 @@
         <v>13</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F7" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="30">
+      <c r="G7" s="29">
         <v>23</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="H7" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="I7" s="32"/>
-      <c r="J7" s="33"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="32"/>
     </row>
     <row r="8" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
       <c r="D8" s="9">
         <v>14</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="F8" s="10"/>
-      <c r="G8" s="30">
+      <c r="G8" s="29">
         <v>24</v>
       </c>
-      <c r="H8" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="I8" s="32"/>
-      <c r="J8" s="33"/>
+      <c r="H8" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="31"/>
+      <c r="J8" s="32"/>
       <c r="AB8" s="3"/>
       <c r="AC8" s="3"/>
     </row>
@@ -823,24 +823,24 @@
         <v>15</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="F9" s="10"/>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36"/>
       <c r="AB9" s="3"/>
       <c r="AC9" s="3"/>
     </row>
     <row r="10" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
       <c r="D10" s="9">
         <v>16</v>
       </c>
@@ -850,7 +850,7 @@
       <c r="F10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="29">
+      <c r="G10" s="28">
         <v>25</v>
       </c>
       <c r="H10" s="18" t="s">
@@ -875,15 +875,15 @@
         <v>17</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F11" s="10"/>
-      <c r="G11" s="28" t="s">
+      <c r="G11" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="28"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
       <c r="AB11" s="3"/>
       <c r="AC11" s="3"/>
     </row>
@@ -902,14 +902,14 @@
         <v>16</v>
       </c>
       <c r="F12" s="10"/>
-      <c r="G12" s="34">
+      <c r="G12" s="33">
         <v>26</v>
       </c>
-      <c r="H12" s="35" t="s">
+      <c r="H12" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
       <c r="AB12" s="3"/>
       <c r="AC12" s="3"/>
     </row>
@@ -940,11 +940,11 @@
         <v>32</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
       <c r="AB14" s="3"/>
       <c r="AC14" s="3"/>
     </row>

</xml_diff>